<commit_message>
Update macierz_iMapServer files with new data
</commit_message>
<xml_diff>
--- a/dane/produkty/macierz_iMapServer.xlsx
+++ b/dane/produkty/macierz_iMapServer.xlsx
@@ -1705,7 +1705,7 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Serwer startuje w kilka minut na dowolnym srodowisku IT. Eliminuje tygodniowe wdrozenia reczne i ryzyko bledow konfiguracyjnych. Latwe przenoszenie miedzy srodowiskami (test -&gt; produkcja).</t>
+          <t>Serwer startuje w kilka minut na dowolnym środowisku IT. Eliminuje tygodniowe wdrożenia ręczne i ryzyko błędów konfiguracyjnych. Łatwe przenoszenie między środowiskami (test -&gt; produkcja).</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Wszystkie ustawienia systemu mozna zmienic w jednym pliku tekstowym - bez angazowania programistow. Upraszcza utrzymanie i przyspiesza reakcje na zmiany wymagan.</t>
+          <t>Wszystkie ustawienia systemu można zmienić w jednym pliku tekstowym — bez angażowania programistów. Upraszcza utrzymanie i przyspiesza reakcję na zmiany wymagań.</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Analitycy i specjalisci GIS moga pisac wlasne skrypty analityczne korzystajac z gotowego, profesjonalnego srodowiska - bez instalowania narzedzi na swoich komputerach.</t>
+          <t>Analitycy i specjaliści GIS mogą pisać własne skrypty analityczne korzystając z gotowego, profesjonalnego środowiska — bez instalowania narzędzi na swoich komputerach.</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Koszt licencji jest przewidywalny i niezalezny od liczby uzytkownikow - firma placi za serwer, nie za kazdego pracownika. Ulatwia planowanie budzetu IT.</t>
+          <t>Koszt licencji jest przewidywalny i niezależny od liczby użytkowników — firma płaci za serwer, nie za każdego pracownika. Ułatwia planowanie budżetu IT.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Dane geograficzne organizacji pozostaja wylacznie na jej wlasnych serwerach. Kluczowe dla urzedow, sluzb i firm z wymogami bezpieczenstwa lub certyfikacja ISO 27001.</t>
+          <t>Dane geograficzne organizacji pozostają wyłącznie na jej własnych serwerach. Kluczowe dla urzędów, służb i firm z wymogami bezpieczeństwa lub certyfikacją ISO 27001.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Uzytkownicy widza mapy generowane dynamicznie - zawsze aktualne, bez koniecznosci recznego odswiezania. Kompatybilne z popularnymi przegladarkami mapowymi (QGIS, ArcGIS Pro).</t>
+          <t>Użytkownicy widzą mapy generowane dynamicznie — zawsze aktualne, bez konieczności ręcznego odświeżania. Kompatybilne z popularnymi przeglądarkami mapowymi (QGIS, ArcGIS Pro).</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Umozliwia edycje danych przestrzennych bezposrednio przez przegladarke lub aplikacje mobilna. Pracownicy terenowi moga aktualizowac dane z tabletu - zmiany od razu widoczne dla calej organizacji.</t>
+          <t>Umożliwia edycję danych przestrzennych bezpośrednio przez przeglądarkę lub aplikację mobilną. Pracownicy terenowi mogą aktualizować dane z tabletu — zmiany od razu widoczne dla całej organizacji.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Mapy w postaci gotowych kafelkow laduja sie blyskawicznie nawet przy duzej liczbie uzytkownikow. Idealne dla portali publicznych z tysiarcami odwiedzajacych dziennie.</t>
+          <t>Mapy w postaci gotowych kafli ładują się błyskawicznie nawet przy dużej liczbie użytkowników. Idealne dla portali publicznych z tysiącami odwiedzających dziennie.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Zdjecia lotnicze i satelitarne dostepne jako usluga - uzytkownicy przegladaja je plynnie, bez pobierania gigabajtow danych na komputer.</t>
+          <t>Zdjęcia lotnicze i satelitarne dostępne jako usługa — użytkownicy przeglądają je płynnie, bez pobierania gigabajtów danych na komputer.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Umozliwia prezentacje i analize danych 3D (budynki, rzezba terenu) bez specjalistycznego oprogramowania - wystarczy przegladarka lub prosta aplikacja.</t>
+          <t>Zdjęcia lotnicze, ortofotomapy i modele terenu przetwarzane na serwerze w chwili wyświetlania — użytkownik widzi obraz z nałożoną analizą (np. cieniowanie terenu, NDVI) bez generowania i przechowywania kopii danych.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Modele trojwymiarowe budynkow i infrastruktury dostepne on-line dla urbanistow, architektow i zarzadcow nieruchomosci.</t>
+          <t>Modele trójwymiarowe budynków i infrastruktury dostępne on-line dla urbanistów, architektów i zarządców nieruchomości.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Umozliwia wykonywanie obliczen geometrycznych (odleglosci, pola, przeciecia) przez zewnetrzne aplikacje - bez kupowania osobnych bibliotek matematycznych.</t>
+          <t>Umożliwia wykonywanie obliczeń geometrycznych (odległości, pola, przecięcia) przez zewnętrzne aplikacje — bez kupowania osobnych bibliotek matematycznych.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Automatyzacja powtarzalnych analiz przestrzennych (np. generowanie raportow, bufory, przeliczenia) bez recznej pracy. Skraca czas realizacji procesow z godzin do minut.</t>
+          <t>Automatyzacja powtarzalnych analiz przestrzennych (np. generowanie raportów, bufory, przeliczenia) bez ręcznej pracy. Skraca czas realizacji procesów z godzin do minut.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Duze zbiory punktow (np. zgloszenia, wypadki, pomiary) automatycznie grupowane w klastry na mapie - czytelny obraz rozkladu zjawisk zamiast chaotycznej chmury punktow.</t>
+          <t>Duże zbiory punktów (np. zgłoszenia, wypadki, pomiary) automatycznie grupowane w klastry na mapie — czytelny obraz rozkładu zjawisk zamiast chaotycznej chmury punktów.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Dane z iMapServer sa dostepne w kazdej aplikacji GIS obslugujacej standard WMS. Brak uzaleznienia od jednego dostawcy oprogramowania.</t>
+          <t>Dane z iMapServer są dostępne w każdej aplikacji GIS obsługującej standard WMS. Brak uzależnienia od jednego dostawcy oprogramowania.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="O17" s="6" t="inlineStr">
         <is>
-          <t>potwierdzone</t>
+          <t>do weryfikacji</t>
         </is>
       </c>
       <c r="P17" s="6" t="inlineStr"/>
@@ -3079,7 +3079,11 @@
       <c r="AT17" s="6" t="inlineStr"/>
       <c r="AU17" s="6" t="inlineStr"/>
       <c r="AV17" s="6" t="inlineStr"/>
-      <c r="AW17" s="6" t="inlineStr"/>
+      <c r="AW17" s="6" t="inlineStr">
+        <is>
+          <t>Potwierdzona wyłącznie wersja 1.3.0 (pl.gispartner.imapserver.wms.version, domyślnie 1.3.0 — configuration/configuration/parameters.md:360). Wersja 1.1.1 nie ma potwierdzenia w bazie wiedzy; brak parametru typu acceptVersions. Plik services-type/wms.md jest pusty (0 B). Do potwierdzenia: czy 1.1.1 jest nadal serwowane.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -3114,7 +3118,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Dane wektorowe pobieralne do zewnetrznych systemow i narzedzi (QGIS, ETL) w standardowym formacie OGC. Integracja z rejestrowymi bazami danych.</t>
+          <t>Dane wektorowe pobieralne do zewnętrznych systemów i narzędzi (QGIS, ETL) w standardowym formacie OGC. Integracja z rejestrowymi bazami danych.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -3138,7 +3142,7 @@
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
-          <t>potwierdzone</t>
+          <t>do weryfikacji</t>
         </is>
       </c>
       <c r="P18" s="6" t="inlineStr"/>
@@ -3174,7 +3178,11 @@
       <c r="AT18" s="6" t="inlineStr"/>
       <c r="AU18" s="6" t="inlineStr"/>
       <c r="AV18" s="6" t="inlineStr"/>
-      <c r="AW18" s="6" t="inlineStr"/>
+      <c r="AW18" s="6" t="inlineStr">
+        <is>
+          <t>WFS jako usługa serwerowa jest w trakcie implementacji: changelog 5.1.2060 (2026-02-02) "pierwsza postać GetFeatures", 5.1.2098 "Początki generowania Capa", 5.1.2106 (2026-02-26) "GetFeature zamiast GetFeatures" — nazwa operacji zmieniona na ostatnim buildzie. Operacja Transaction i numer wersji protokołu nie mają potwierdzenia (brak parametru wfs.version; sekcja OGC w parameters.md zawiera tylko WMTS, WMS i WPS). WFS jako źródło danych (IMS-5.2.07) pozostaje potwierdzony. Do potwierdzenia: zakres operacji i wersja protokołu w wersji wydanej.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -3209,7 +3217,7 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Gotowe kafelki w standardzie WMTS - kompatybilne z QGIS, ArcGIS, OpenLayers i wszystkimi popularnymi narzedzami GIS bez zadnej konfiguracji.</t>
+          <t>Gotowe kafle w standardzie WMTS — kompatybilne z QGIS, ArcGIS, OpenLayers i wszystkimi popularnymi narzędziami GIS bez żadnej konfiguracji.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -3308,7 +3316,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Nowoczesne, RESTowe API do danych przestrzennych - kompatybilne z najnowszymi standardami europejskimi (INSPIRE) i wymaganiami srodowisk cloud-native.</t>
+          <t>Nowoczesne, RESTowe API do danych przestrzennych — kompatybilne z najnowszymi standardami europejskimi (INSPIRE) i wymaganiami środowisk cloud-native.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -3403,7 +3411,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Mozliwosc zadawania precyzyjnych pytan o dane (np. dzialki pow. &gt; 1 ha w gminie X) w zrozumialym jezyku. Nie wymaga pisania SQL przez uzytkownika koncowego.</t>
+          <t>Możliwość zadawania precyzyjnych pytań o dane (np. działki pow. &gt; 1 ha w gminie X) w zrozumiałym języku. Nie wymaga pisania SQL przez użytkownika końcowego.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -3498,7 +3506,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Zaawansowane filtrowanie danych: po geometrii, atrybutach, czasie, statystykach - w jednym zadaniu. Mniej zapytan do serwera = szybsze aplikacje.</t>
+          <t>Zaawansowane filtrowanie danych: po geometrii, atrybutach, czasie, statystykach — w jednym zadaniu. Mniej zapytań do serwera = szybsze aplikacje.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -3593,7 +3601,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Mozliwosc precyzyjnego okreslenia topologicznych relacji przestrzennych miedzy obiektami (np. czy granica dzialki A dotyka granicy dzialki B). Przydatne w kontrolach jakosci danych.</t>
+          <t>Możliwość precyzyjnego określenia topologicznych relacji przestrzennych między obiektami (np. czy granica działki A dotyka granicy działki B). Przydatne w kontrolach jakości danych.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -3688,7 +3696,7 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Mozliwosc przegladania danych wedlug stanu na dowolna date w przeszlosci - bez duplikowania bazy danych. Kluczowe dla ewidencji, gdzie historia zmian jest wymagana prawnie.</t>
+          <t>Możliwość przeglądania danych według stanu na dowolną datę w przeszłości — bez duplikowania bazy danych. Kluczowe dla ewidencji, gdzie historia zmian jest wymagana prawnie.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -3783,7 +3791,7 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Tworzenie wyliczanych pol (np. wskaznik zabudowy, pelny adres z osobnych kolumn) bez modyfikowania struktury bazy danych. Oszczedza czas i eliminuje ryzyko bledow migracji.</t>
+          <t>Tworzenie wyliczanych pól (np. wskaźnik zabudowy, pełny adres z osobnych kolumn) bez modyfikowania struktury bazy danych. Oszczędza czas i eliminuje ryzyko błędów migracji.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -3878,7 +3886,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Wyniki zapytan mozna zwrocic od razu ze stylem graficznym (kolor, grubosc linii) - aplikacje klienckie nie musza samodzielnie definiowac symboliki.</t>
+          <t>Wyniki zapytań można zwrócić od razu ze stylem graficznym (kolor, grubość linii) — aplikacje klienckie nie muszą samodzielnie definiować symboliki.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
@@ -3973,7 +3981,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Filtrowanie zagregowanych wynikow (np. tylko gminy, gdzie suma powierzchni &gt; 1000 ha) w jednym zapytaniu - zastepuje przetwarzanie po stronie klienta.</t>
+          <t>Filtrowanie zagregowanych wyników (np. tylko gminy, gdzie suma powierzchni &gt; 1000 ha) w jednym zapytaniu — zastępuje przetwarzanie po stronie klienta.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
@@ -4068,7 +4076,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Operacje na zbiorach danych (suma, iloczyn, roznica) - np. obiekty wspolne dla dwoch warstw. Eliminuje reczne porownywanie w tabelkach.</t>
+          <t>Operacje na zbiorach danych (suma, iloczyn, różnica) — np. obiekty wspólne dla dwóch warstw. Eliminuje ręczne porównywanie w tabelkach.</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
@@ -4163,7 +4171,7 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Eksport widoku mapy jako obrazu rastrowego do dokumentow, prezentacji i raportow. Formatowanie gotowe do druku.</t>
+          <t>Eksport widoku mapy jako obrazu rastrowego do dokumentów, prezentacji i raportów. Formatowanie gotowe do druku.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
@@ -4258,7 +4266,7 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>Klikniecie punktu na mapie zwraca atrybuty wszystkich obiektow w tym miejscu - podstawa kazdej interaktywnej aplikacji mapowej.</t>
+          <t>Klikniecie punktu na mapie zwraca atrybuty wszystkich obiektów w tym miejscu — podstawa każdej interaktywnej aplikacji mapowej.</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
@@ -4353,7 +4361,7 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Eksport danych do SQLite (offline dla aplikacji mobilnych), GeoPackage, modeli 3D (GLB/OBJ) bez koniecznosci korzystania z osobnych narzedzi konwersji.</t>
+          <t>Eksport danych do SQLite (offline dla aplikacji mobilnych), GeoPackage, modeli 3D (GLB/OBJ) bez konieczności korzystania z osobnych narzędzi konwersji.</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
@@ -4448,7 +4456,7 @@
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Administratorzy moga tworzyc, modyfikowac i usuwac konfiguracje map przez API - automatyzacja zarzadzania bez logowania do panelu.</t>
+          <t>Administratorzy mogą tworzyć, modyfikować i usuwać konfiguracje map przez API — automatyzacja zarządzania bez logowania do panelu.</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
@@ -4543,7 +4551,7 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>Automatyczne generowanie kafelkow na zadanie - zawsze aktualne bez recznego odbudowywania cache.</t>
+          <t>Automatyczne generowanie kafli na zadanie — zawsze aktualne bez ręcznego odbudowywania cache.</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
@@ -4638,7 +4646,7 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Przejrzysty podzial na bazy, schematy i tabele - administratorzy widza cala strukture danych w jednym miejscu i moga zarzadzac uprawnieniami na kazdym poziomie.</t>
+          <t>Przejrzysty podział na bazy, schematy i tabele — administratorzy widzą cala strukturę danych w jednym miejscu i mogą zarządzać uprawnieniami na każdym poziomie.</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
@@ -4733,7 +4741,7 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Bezposrednie odpytywanie tabel bazodanowych przez API - umozliwia budowanie raportow i integracji bez tworzenia osobnych widokow w uslugach mapowych.</t>
+          <t>Bezpośrednie odpytywanie tabel bazodanowych przez API — umożliwia budowanie raportów i integracji bez tworzenia osobnych widoków w usługach mapowych.</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
@@ -4828,7 +4836,7 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Pelna edycja danych (dodawanie, aktualizacja, usuwanie obiektow) przez bezpieczne API - bez bezposredniego dostepu do bazy danych przez uzytkownika.</t>
+          <t>Pełna edycja danych (dodawanie, aktualizacja, usuwanie obiektów) przez bezpieczne API — bez bezpośredniego dostępu do bazy danych przez użytkownika.</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
@@ -4923,7 +4931,7 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Masowe przeliczenie wartosci atrybutow (np. aktualizacja pola status dla tysiecy rekordow) w jednej operacji - bez recznej edycji.</t>
+          <t>Masowe przeliczenie wartości atrybutów (np. aktualizacja pola status dla tysięcy rekordów) w jednej operacji — bez ręcznej edycji.</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
@@ -5018,7 +5026,7 @@
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>Dodawanie nowych pol do tabel przez API bez interwencji administratora bazy danych - przyspiesza rozwoj systemu.</t>
+          <t>Dodawanie nowych pol do tabel przez API bez interwencji administratora bazy danych — przyspiesza rozwój systemu.</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
@@ -5113,7 +5121,7 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Definiowanie powiazan miedzy tabelami (np. dzialka &lt;-&gt; wlasciciel) - dane powiazane dostepne w jednym zapytaniu.</t>
+          <t>Definiowanie powiązań między tabelami (np. działka &lt;-&gt; właściciel) — dane powiązane dostępne w jednym zapytaniu.</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
@@ -5208,7 +5216,7 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Tworzenie logicznych widokow na dane (np. tylko aktywne obiekty danego uzytkownika) bez tworzenia kopii fizycznych danych.</t>
+          <t>Tworzenie logicznych widoków na dane (np. tylko aktywne obiekty danego użytkownika) bez tworzenia kopii fizycznych danych.</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
@@ -5303,7 +5311,7 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Automatyczne sledzenie historii zmian w tabeli - kazda modyfikacja zapisywana z data. Spelnienie wymogan prawnych (ewidencje, audyty) bez dodatkowych rozwiazan.</t>
+          <t>Automatyczne śledzenie historii zmian w tabeli — każda modyfikacja zapisywana z data. Spełnienie wymogan prawnych (ewidencje, audyty) bez dodatkowych rozwiązań.</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
@@ -5398,7 +5406,7 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>Przechowywanie i serwowanie plikow (zdjecia, dokumenty, skany) powiazanych z obiektami przestrzennymi - kompletna dokumentacja w jednym miejscu.</t>
+          <t>Przechowywanie i serwowanie plików (zdjęcia, dokumenty, skany) powiązanych z obiektami przestrzennymi — kompletna dokumentacja w jednym miejscu.</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
@@ -5493,7 +5501,7 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>Listy dopuszczalnych wartosci dla pol (np. typy uzytkow gruntowych) zarzadzane centralnie - spojnosc i poprawnosc danych we wszystkich aplikacjach.</t>
+          <t>Listy dopuszczalnych wartości dla pol (np. typy użytków gruntowych) zarządzane centralnie — spójność i poprawność danych we wszystkich aplikacjach.</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
@@ -5588,7 +5596,7 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>Przyspieszenie zapytan przestrzennych przez indeksy - uzytkownik otrzymuje wyniki w sekundy nawet dla milionow obiektow.</t>
+          <t>Przyspieszenie zapytań przestrzennych przez indeksy — użytkownik otrzymuje wyniki w sekundy nawet dla milionów obiektów.</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
@@ -5683,7 +5691,7 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>Zabezpieczenie danych przed rownoczesna edycja przez wielu uzytkownikow - eliminacja nadpisywania zmian w srodowiskach wielouzytkownikowych.</t>
+          <t>Zabezpieczenie danych przed równoczesną edycją przez wielu użytkowników — eliminacja nadpisywania zmian w środowiskach wieloużytkownikowych.</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
@@ -5778,7 +5786,7 @@
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>Precyzyjne zarzadzanie kluczami glownymi i identyfikatorami - spojnosc danych przy integracji z zewnetrznymi systemami (GML, EGiB, EMUiA).</t>
+          <t>Precyzyjne zarządzanie kluczami głównymi i identyfikatorami — spójność danych przy integracji z zewnętrznymi systemami (GML, EGiB, EMUiA).</t>
         </is>
       </c>
       <c r="H46" s="6" t="inlineStr">
@@ -5873,7 +5881,7 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>Mozliwosc definiowania wlasnych funkcji obliczeniowych (np. obliczenie klasy bonitacji, przeliczenie podatku) dostepnych we wszystkich zapytaniach.</t>
+          <t>Możliwość definiowania własnych funkcji obliczeniowych (np. obliczenie klasy bonitacji, przeliczenie podatku) dostępnych we wszystkich zapytaniach.</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
@@ -5968,7 +5976,7 @@
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>Utrzymanie porzadku w bazie danych przez usuwanie nieuzywanych tabel i schematow - bez bezposredniego dostepu do silnika bazy danych.</t>
+          <t>Utrzymanie porządku w bazie danych przez usuwanie nieużywanych tabel i schematów — bez bezpośredniego dostępu do silnika bazy danych.</t>
         </is>
       </c>
       <c r="H48" s="6" t="inlineStr">
@@ -6063,7 +6071,7 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>Jedno, spojne API REST obsluguje wszystkie funkcje systemu - integracja z dowolnym systemem informatycznym (ERP, CRM, portale) przez standardowe wywolania HTTP.</t>
+          <t>Jedno, spojne API REST obsługuje wszystkie funkcje systemu — integracja z dowolnym systemem informatycznym (ERP, CRM, portale) przez standardowe wywołania HTTP.</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
@@ -6158,7 +6166,7 @@
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>Wyszukiwanie obiektow na mapie po atrybutach i lokalizacji - fundament kazdej aplikacji GIS dla uzytkownikow koncowych.</t>
+          <t>Wyszukiwanie obiektów na mapie po atrybutach i lokalizacji — fundament każdej aplikacji GIS dla użytkowników końcowych.</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
@@ -6253,7 +6261,7 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>Pobieranie duzych zbiorow danych stronami - aplikacje laduja dane plynnie bez przeciazania serwera i klienta.</t>
+          <t>Pobieranie dużych zbiorów danych stronami — aplikacje ładują dane płynnie bez przeciążania serwera i klienta.</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
@@ -6348,7 +6356,7 @@
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Wyliczanie wartosci na biezaco (np. pelny adres z osobnych pol, wskazniki finansowe) - bez koniecznosci modyfikowania struktury bazy.</t>
+          <t>Wyliczanie wartości na bieżąco (np. pełny adres z osobnych pól, wskaźniki finansowe) — bez konieczności modyfikowania struktury bazy.</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
@@ -6443,7 +6451,7 @@
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>Jeden klik na mapie moze pobrac dane powiazane z obiektem (np. klikniecie dzialki -&gt; lista wlascicieli, historia transakcji) - bez kolejnych recznych wyszukan.</t>
+          <t>Jeden klik na mapie może pobrać dane powiązane z obiektem (np. klikniecie działki -&gt; lista właścicieli, historia transakcji) — bez kolejnych ręcznych wyszukań.</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
@@ -6538,7 +6546,7 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Logiczne widoki na dane (np. tylko moje zadania, aktywne zgloszenia) bez tworzenia osobnych tabel - kazdy uzytkownik widzi to, czego potrzebuje.</t>
+          <t>Logiczne widoki na dane (np. tylko moje zadania, aktywne zgłoszenia) bez tworzenia osobnych tabel — każdy użytkownik widzi to, czego potrzebuje.</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr">
@@ -6633,7 +6641,7 @@
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>Kazdy uzytkownik automatycznie widzi tylko swoje dane lub dane swojej organizacji - bezpieczenstwo i prywatnosc bez rozbudowanej logiki w aplikacji klienckiej.</t>
+          <t>Każdy użytkownik automatycznie widzi tylko swoje dane lub dane swojej organizacji — bezpieczeństwo i prywatność bez rozbudowanej logiki w aplikacji klienckiej.</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
@@ -6728,7 +6736,7 @@
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>Automatyczne wypelnianie pol na podstawie wczesniej wprowadzonych danych - przyspiesza prace edytorow danych terenowych.</t>
+          <t>Automatyczne wypełnianie pol na podstawie wcześniej wprowadzonych danych — przyspiesza pracę edytorów danych terenowych.</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr">
@@ -6823,7 +6831,7 @@
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>Przechowywanie i udostepnianie obrazow, dokumentow i innych plikow binarnych bezposrednio w tabeli przestrzennej.</t>
+          <t>Przechowywanie i udostępnianie obrazów, dokumentów i innych plików binarnych bezpośrednio w tabeli przestrzennej.</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr">
@@ -6918,7 +6926,7 @@
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>Opisy pol i aliasy dostepne w kilku jezykach - system GIS obsluguje wielojezyczne organizacje bez duplikowania konfiguracji.</t>
+          <t>Opisy pol i aliasy dostępne w kilku językach — system GIS obsługuje wielojęzyczne organizacje bez duplikowania konfiguracji.</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr">
@@ -7013,7 +7021,7 @@
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>Slowniki wartosci dozwolonych (np. typy drog, klasy budynkow) zarzadzane centralnie - poprawiaja jakosc danych i ulatwiaja raportowanie.</t>
+          <t>Słowniki wartości dozwolonych (np. typy dróg, klasy budynków) zarządzane centralnie — poprawiają jakość danych i ułatwiają raportowanie.</t>
         </is>
       </c>
       <c r="H59" s="6" t="inlineStr">
@@ -7108,7 +7116,7 @@
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>Bezpieczna komunikacja HTTPS i uwierzytelnianie tokenami JWT - standard bezpieczenstwa dla aplikacji webowych i mobilnych.</t>
+          <t>Bezpieczna komunikacja HTTPS i uwierzytelnianie tokenami JWT (OAuth 2.0) na poziomie API — integracja z aplikacjami webowymi i mobilnymi bez przesyłania danych logowania przy każdym żądaniu.</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr">
@@ -7203,7 +7211,7 @@
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>Administratorzy moga publikowac, aktualizowac i wycofywac aplikacje webowe z jednego miejsca - bez angazowania dzialu IT do kazdej zmiany.</t>
+          <t>Administratorzy mogą publikować, aktualizować i wycofywać aplikacje webowe z jednego miejsca — bez angażowania działu IT do każdej zmiany.</t>
         </is>
       </c>
       <c r="H61" s="6" t="inlineStr">
@@ -7298,7 +7306,7 @@
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>Pelna edycja konfiguracji aplikacji webowych przez API - automatyzacja wdrozen i aktualizacji.</t>
+          <t>Pełna edycja konfiguracji aplikacji webowych przez API — automatyzacja wdrożeń i aktualizacji.</t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr">
@@ -7393,7 +7401,7 @@
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>Kontrola kto moze korzystac z ktorych aplikacji - bezpieczne srodowisko wieloorganizacyjne (np. kilka wydzialow, kilka klientow).</t>
+          <t>Kontrola kto może korzystać z których aplikacji — bezpieczne środowisko wieloorganizacyjne (np. kilka wydziałów, kilka klientów).</t>
         </is>
       </c>
       <c r="H63" s="6" t="inlineStr">
@@ -7488,7 +7496,7 @@
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>Miniatura podgladu aplikacji widoczna w katalogu zasobow - uzytkownicy latwo odnajduja wlasciwa aplikacje bez otwierania kazdej z osobna.</t>
+          <t>Miniatura podglądu aplikacji widoczna w katalogu zasobów — użytkownicy łatwo odnajdują właściwa aplikacje bez otwierania każdej z osobną.</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr">
@@ -7583,7 +7591,7 @@
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>Mozliwosc rozszerzenia systemu o niestandardowe operacje analityczne napisane przez dzial IT w Javie - system rosnie razem z potrzebami organizacji.</t>
+          <t>Możliwość rozszerzenia systemu o niestandardowe operacje analityczne napisane przez dział IT w Javie — system rośnie razem z potrzebami organizacji.</t>
         </is>
       </c>
       <c r="H65" s="6" t="inlineStr">
@@ -7678,7 +7686,7 @@
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>Analitycy GIS moga pisac skrypty w Pythonie i uruchamiac je jako uslugi serwerowe - gotowe srodowisko, brak konfiguracji.</t>
+          <t>Analitycy GIS mogą pisać skrypty w Pythonie i uruchamiać je jako usługi serwerowe — gotowe środowisko, brak konfiguracji.</t>
         </is>
       </c>
       <c r="H66" s="6" t="inlineStr">
@@ -7773,7 +7781,7 @@
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>Zlozone analizy wieloetapowe (np. bufor -&gt; selekcja -&gt; statystyki -&gt; eksport) definiowane raz, uruchamiane automatycznie - eliminacja recznej pracy powtarzalnej.</t>
+          <t>Złożone analizy wieloetapowe (np. bufor -&gt; selekcja -&gt; statystyki -&gt; eksport) definiowane raz, uruchamiane automatycznie — eliminacja ręcznej pracy powtarzalnej.</t>
         </is>
       </c>
       <c r="H67" s="6" t="inlineStr">
@@ -7868,7 +7876,7 @@
       </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>Analizy uruchamiane automatycznie o zadanej porze (np. codziennie o 6:00 generuje raport dla zarzadu) - bez recznego uruchamiania przez pracownika.</t>
+          <t>Analizy uruchamiane automatycznie o zadanej porze (np. codziennie o 6:00 generuje raport dla zarządu) — bez ręcznego uruchamiania przez pracownika.</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr">
@@ -7963,7 +7971,7 @@
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>Proste analizy dzialaja natychmiast (odpowiedz w sekundy). Zlozone obliczenia dzialaja w tle - uzytkownik nie czeka i moze wykonywac inne czynnosci.</t>
+          <t>Proste analizy działają natychmiast (odpowiedz w sekundy). Złożone obliczenia działają w tle — użytkownik nie czeka i może wykonywać inne czynności.</t>
         </is>
       </c>
       <c r="H69" s="6" t="inlineStr">
@@ -8058,7 +8066,7 @@
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>Tworzenie stref buforowych (zasieg oddzialywania), wyznaczanie srodkow ciezkosci obiektow, obliczanie dlugosci i powierzchni - podstawowe operacje analityczne.</t>
+          <t>Tworzenie stref buforowych (zasięg oddziaływania), wyznaczanie środków ciężkości obiektów, obliczanie długości i powierzchni — podstawowe operacje analityczne.</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr">
@@ -8153,7 +8161,7 @@
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>Upraszczanie ksztaltow obiektow, podzial linii na rowne odcinki, dzielenie duzych poligonow - operacje przygotowania danych.</t>
+          <t>Upraszczanie kształtów obiektów, podział linii na równe odcinki, dzielenie dużych poligonów — operacje przygotowania danych.</t>
         </is>
       </c>
       <c r="H71" s="6" t="inlineStr">
@@ -8248,7 +8256,7 @@
       </c>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>Rozbijanie obiektow wieloczesciowych na skladowe, ekstrakcja wierzcholkow, wyrownywanie do siatki - narzedzia kontroli jakosci geometrii.</t>
+          <t>Rozbijanie obiektów wieloczęściowych na składowe, ekstrakcja wierzchołków, wyrównywanie do siatki — narzędzia kontroli jakości geometrii.</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">
@@ -8343,7 +8351,7 @@
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>Obroty, skalowanie, przesuniecia geometrii oraz transformacje miedzy ukladami wspolrzednych - przygotowanie danych do integracji i kartowania.</t>
+          <t>Obroty, skalowanie, przesunięcia geometrii oraz transformacje między układami współrzędnych — przygotowanie danych do integracji i kartowania.</t>
         </is>
       </c>
       <c r="H73" s="6" t="inlineStr">
@@ -8438,7 +8446,7 @@
       </c>
       <c r="G74" s="6" t="inlineStr">
         <is>
-          <t>Minimalne okragi opisane, generowanie siatek punktow probkowania, importowanie punktow z list CSV - narzedzia planowania pomiarow i inwentaryzacji.</t>
+          <t>Minimalne okręgi opisane, generowanie siatek punktów próbkowania, importowanie punktów z list CSV — narzędzia planowania pomiarów i inwentaryzacji.</t>
         </is>
       </c>
       <c r="H74" s="6" t="inlineStr">
@@ -8533,7 +8541,7 @@
       </c>
       <c r="G75" s="6" t="inlineStr">
         <is>
-          <t>Obliczanie przeciecia, roznicy i sumy zbiorow obiektow przestrzennych - np. ktore dzialki NIE leza w zadnej strefie ochronnej.</t>
+          <t>Obliczanie przecięcia, różnicy i sumy zbiorów obiektów przestrzennych — np. które działki NIE leżą w żadnej strefie ochronnej.</t>
         </is>
       </c>
       <c r="H75" s="6" t="inlineStr">
@@ -8628,7 +8636,7 @@
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>Scalanie wielu obiektow w jeden (np. wszystkie odcinki drogi w jedna calosc), kopiowanie danych miedzy warstwami.</t>
+          <t>Scalanie wielu obiektów w jeden (np. wszystkie odcinki drogi w jedna całość), kopiowanie danych między warstwami.</t>
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr">
@@ -8723,7 +8731,7 @@
       </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t>Usuwanie zbednych obiektow wedlug atrybutow lub lokalizacji - czyszczenie i odchudzanie zbiorow danych.</t>
+          <t>Usuwanie zbędnych obiektów według atrybutów lub lokalizacji — czyszczenie i odchudzanie zbiorów danych.</t>
         </is>
       </c>
       <c r="H77" s="6" t="inlineStr">
@@ -8818,7 +8826,7 @@
       </c>
       <c r="G78" s="6" t="inlineStr">
         <is>
-          <t>Automatyczne przypisywanie atrybutow z jednej warstwy do drugiej na podstawie lokalizacji (np. dodanie nazwy gminy do kazdego punktu adresowego).</t>
+          <t>Automatyczne przypisywanie atrybutów z jednej warstwy do drugiej na podstawie lokalizacji (np. dodanie nazwy gminy do każdego punktu adresowego).</t>
         </is>
       </c>
       <c r="H78" s="6" t="inlineStr">
@@ -8913,7 +8921,7 @@
       </c>
       <c r="G79" s="6" t="inlineStr">
         <is>
-          <t>Obliczanie statystyk (suma, srednia, min, max) per obszar lub kategoria - np. laczna powierzchnia uzytkow rolnych per powiat.</t>
+          <t>Obliczanie statystyk (suma, średnia, min, max) per obszar lub kategoria — np. łączna powierzchnia użytków rolnych per powiat.</t>
         </is>
       </c>
       <c r="H79" s="6" t="inlineStr">
@@ -9008,7 +9016,7 @@
       </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>Analiza gestosci zjawisk, wykrywanie skupisk (hot-spots), wyznaczanie najblizszego sasiada, generowanie diagramow Woronoja.</t>
+          <t>Analiza gęstości zjawisk, wykrywanie skupisk (hot-spots), wyznaczanie najbliższego sąsiada, generowanie diagramów Woronoja.</t>
         </is>
       </c>
       <c r="H80" s="6" t="inlineStr">
@@ -9103,7 +9111,7 @@
       </c>
       <c r="G81" s="6" t="inlineStr">
         <is>
-          <t>Zamiana adresow na wspolrzedne geograficzne z uzyciem Nominatim/OpenStreetMap - lokalizowanie obiektow na mapie na podstawie adresu tekstowego.</t>
+          <t>Zamiana adresów na współrzędne geograficzne z użyciem Nominatim/OpenStreetMap — lokalizowanie obiektów na mapie na podstawie adresu tekstowego.</t>
         </is>
       </c>
       <c r="H81" s="6" t="inlineStr">
@@ -9198,7 +9206,7 @@
       </c>
       <c r="G82" s="6" t="inlineStr">
         <is>
-          <t>Generowanie map cieniowania (widocznosc uksztaltowania terenu), map nachylen zboczy, wycinanie obszarow z rastrow - podstawowe analizy terenowe.</t>
+          <t>Generowanie map cieniowania (widoczność ukształtowania terenu), map nachyleń zboczy, wycinanie obszarów z rastrów — podstawowe analizy terenowe.</t>
         </is>
       </c>
       <c r="H82" s="6" t="inlineStr">
@@ -9293,7 +9301,7 @@
       </c>
       <c r="G83" s="6" t="inlineStr">
         <is>
-          <t>Konwersja danych rastrowych (np. ortofoto, NMT) na wektory i odwrotnie - przygotowanie danych do analiz lub wizualizacji.</t>
+          <t>Konwersja danych rastrowych (np. ortofoto, NMT) na wektory i odwrotnie — przygotowanie danych do analiz lub wizualizacji.</t>
         </is>
       </c>
       <c r="H83" s="6" t="inlineStr">
@@ -9388,7 +9396,7 @@
       </c>
       <c r="G84" s="6" t="inlineStr">
         <is>
-          <t>Laczenie wielu rastrow w jeden, obliczanie statystyk na rastrze (np. srednia wysokosc), analiza pokrycia terenu.</t>
+          <t>Łączenie wielu rastrów w jeden, obliczanie statystyk na rastrze (np. średnia wysokość), analiza pokrycia terenu.</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
@@ -9483,7 +9491,7 @@
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
-          <t>Import danych z roznych formatow i eksport do wielu formatow - integracja z zewnetrznymi dostawcami danych (GUGiK, BDOT, OSM).</t>
+          <t>Import danych z różnych formatów i eksport do wielu formatów — integracja z zewnętrznymi dostawcami danych (GUGiK, BDOT, OSM).</t>
         </is>
       </c>
       <c r="H85" s="6" t="inlineStr">
@@ -9578,7 +9586,7 @@
       </c>
       <c r="G86" s="6" t="inlineStr">
         <is>
-          <t>Tworzenie, modyfikacja i usuwanie tabel i schematow bazodanowych przez API - pelne zarzadzanie struktura danych bez narzedzi bazodanowych.</t>
+          <t>Tworzenie, modyfikacja i usuwanie tabel i schematów bazodanowych przez API — pełne zarządzanie struktura danych bez narzędzi bazodanowych.</t>
         </is>
       </c>
       <c r="H86" s="6" t="inlineStr">
@@ -9673,7 +9681,7 @@
       </c>
       <c r="G87" s="6" t="inlineStr">
         <is>
-          <t>Zarzadzanie kolekcjami zdiec lotniczych i satelitarnych (mozaiki) oraz trojwymiarowymi modelami terenu i budynkow.</t>
+          <t>Zarządzanie kolekcjami zdjęć lotniczych i satelitarnych (mozaiki) oraz trójwymiarowymi modelami terenu i budynków.</t>
         </is>
       </c>
       <c r="H87" s="6" t="inlineStr">
@@ -9768,7 +9776,7 @@
       </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>Wizualizacja danych rastrowych w roznych skalach kolorow (gradienty, klasyfikacje) - np. mapa temperatur, poziomow halasu, zagrozen powodziowych.</t>
+          <t>Wizualizacja danych rastrowych w różnych skalach kolorów (gradienty, klasyfikacje) — np. mapa temperatur, poziomów hałasu, zagrożeń powodziowych.</t>
         </is>
       </c>
       <c r="H88" s="6" t="inlineStr">
@@ -9859,7 +9867,7 @@
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>Przetwarzanie rastrow w locie: zmiana kontrastu, wyostrzanie, NDVI, kompozyty - uzytkownik widzi przetworzone obrazy bez generowania kopii.</t>
+          <t>Przetwarzanie rastrów w locie: zmiana kontrastu, wyostrzanie, NDVI, kompozyty — użytkownik widzi przetworzone obrazy bez generowania kopii.</t>
         </is>
       </c>
       <c r="H89" s="6" t="inlineStr">
@@ -9950,7 +9958,7 @@
       </c>
       <c r="G90" s="6" t="inlineStr">
         <is>
-          <t>Pre-generowane kafelki rastrowe (zdjecia lotnicze, mapy topograficzne) serwowane blyskawicznie przy duzym obciazeniu.</t>
+          <t>Pre-generowane kafle rastrowe (zdjęcia lotnicze, mapy topograficzne) serwowane błyskawicznie przy dużym obciążeniu.</t>
         </is>
       </c>
       <c r="H90" s="6" t="inlineStr">
@@ -10041,7 +10049,7 @@
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
-          <t>Obsluga ponad 200 formatow i ukladow danych rastrowych - czytanie danych z dowolnego zrodla bez konwersji wstepnej.</t>
+          <t>Obsługa ponad 200 formatów i układów danych rastrowych — czytanie danych z dowolnego źródła bez konwersji wstępnej.</t>
         </is>
       </c>
       <c r="H91" s="6" t="inlineStr">
@@ -10132,7 +10140,7 @@
       </c>
       <c r="G92" s="6" t="inlineStr">
         <is>
-          <t>Automatyczne upraszczanie i agregowanie danych rastrowych dla mniejszych skal - mapa wyglada czytelnie na kazdym poziomie przyblizenia.</t>
+          <t>Automatyczne upraszczanie i agregowanie danych rastrowych dla mniejszych skal — mapa wygląda czytelnie na każdym poziomie przybliżenia.</t>
         </is>
       </c>
       <c r="H92" s="6" t="inlineStr">
@@ -10223,7 +10231,7 @@
       </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t>Zarzadzanie cache rastrowym przez API: czyszczenie, odbudowa, monitorowanie - automatyzacja konserwacji bez recznej interwencji.</t>
+          <t>Zarządzanie cache rastrowym przez API: czyszczenie, odbudowa, monitorowanie — automatyzacja konserwacji bez ręcznej interwencji.</t>
         </is>
       </c>
       <c r="H93" s="6" t="inlineStr">
@@ -10314,7 +10322,7 @@
       </c>
       <c r="G94" s="6" t="inlineStr">
         <is>
-          <t>Dane przestrzenne przechowywane w wiodacej open-source bazie GIS. Pelna obsluga zaawansowanej geometrii, analiz i replikacji.</t>
+          <t>Dane przestrzenne przechowywane w wiodącej open-source bazie GIS. Pełna obsługa zaawansowanej geometrii, analiz i replikacji.</t>
         </is>
       </c>
       <c r="H94" s="6" t="inlineStr">
@@ -10405,7 +10413,7 @@
       </c>
       <c r="G95" s="6" t="inlineStr">
         <is>
-          <t>Integracja z Oracle - standardowa baza danych w duzych organizacjach korporacyjnych i administracji publicznej. Obie geometrie Oracle natywnie wspierane.</t>
+          <t>Integracja z Oracle — standardowa baza danych w dużych organizacjach korporacyjnych i administracji publicznej. Obie geometrie Oracle natywnie wspierane.</t>
         </is>
       </c>
       <c r="H95" s="6" t="inlineStr">
@@ -10496,7 +10504,7 @@
       </c>
       <c r="G96" s="6" t="inlineStr">
         <is>
-          <t>Automatyczne filtrowanie danych na poziomie bazy - rozni uzytkownicy widza rozne podzbiory tych samych tabel (np. dane tylko swojej gminy). Bezpieczenstwo bez logiki w aplikacji.</t>
+          <t>Automatyczne filtrowanie danych na poziomie bazy — różni użytkownicy widzą różne podzbiory tych samych tabel (np. dane tylko swojej gminy). Bezpieczeństwo bez logiki w aplikacji.</t>
         </is>
       </c>
       <c r="H96" s="6" t="inlineStr">
@@ -10587,7 +10595,7 @@
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
-          <t>Integracja z Microsoft SQL Server i Active Directory (NTLM) - uzytkownicy loguja sie do systemu GIS tymi samymi danymi co do komputera sluzbowego.</t>
+          <t>Integracja z Microsoft SQL Server i Active Directory (NTLM) — użytkownicy logują się do systemu GIS tymi samymi danymi co do komputera służbowego.</t>
         </is>
       </c>
       <c r="H97" s="6" t="inlineStr">
@@ -10678,7 +10686,7 @@
       </c>
       <c r="G98" s="6" t="inlineStr">
         <is>
-          <t>Lekka baza plikowa (jeden plik) - idealna do dystrybucji danych w terenie (inspektorzy, tablety) i jako format wymiany offline.</t>
+          <t>Lekka baza w jednym pliku jako źródło danych — wdrożenia bez serwera bazodanowego oraz praca w terenie bez łącza.</t>
         </is>
       </c>
       <c r="H98" s="6" t="inlineStr">
@@ -10769,7 +10777,7 @@
       </c>
       <c r="G99" s="6" t="inlineStr">
         <is>
-          <t>Analityczna baza danych DuckDB jako zrodlo - umozliwia analize bardzo duzych zbiorow tabelarycznych bez osobnej hurtowni danych.</t>
+          <t>Analityczna baza danych DuckDB jako źródło — umożliwia analizę bardzo dużych zbiorów tabelarycznych bez osobnej hurtowni danych.</t>
         </is>
       </c>
       <c r="H99" s="6" t="inlineStr">
@@ -10860,7 +10868,7 @@
       </c>
       <c r="G100" s="6" t="inlineStr">
         <is>
-          <t>Dane z zewnetrznych serwisow WFS (np. GUGIK, EMUiA, BDOT) dostepne jako warstwy mapy - aktualne dane bez kopiowania do lokalnej bazy.</t>
+          <t>Dane z zewnętrznych serwisów WFS (np. GUGIK, EMUiA, BDOT) dostępne jako warstwy mapy — aktualne dane bez kopiowania do lokalnej bazy.</t>
         </is>
       </c>
       <c r="H100" s="6" t="inlineStr">
@@ -10951,7 +10959,7 @@
       </c>
       <c r="G101" s="6" t="inlineStr">
         <is>
-          <t>Nowoczesne zewnetrzne API (np. europejskie rejestry INSPIRE) jako zywe zrodlo danych - zawsze aktualne dane bez lokalnej kopii.</t>
+          <t>Nowoczesne zewnętrzne API (np. europejskie rejestry INSPIRE) jako żywe źródło danych — zawsze aktualne dane bez lokalnej kopii.</t>
         </is>
       </c>
       <c r="H101" s="6" t="inlineStr">
@@ -11042,7 +11050,7 @@
       </c>
       <c r="G102" s="6" t="inlineStr">
         <is>
-          <t>Mozliwosc korzystania z plikow Geodatabase (format Esri) jako zrodla danych - ulatwia migracje z dotychczasowego srodowiska ArcGIS.</t>
+          <t>Możliwość korzystania z plików Geodatabase (format Esri) jako źródła danych — ułatwia migracje z dotychczasowego środowiska ArcGIS.</t>
         </is>
       </c>
       <c r="H102" s="6" t="inlineStr">
@@ -11133,7 +11141,7 @@
       </c>
       <c r="G103" s="6" t="inlineStr">
         <is>
-          <t>Zewnetrzne uslugi WMS (np. mapa zasadnicza, ortofoto z geoportal.gov.pl) jako warstwy tla w mapach - bez pobierania danych.</t>
+          <t>Zewnętrzne usługi WMS (np. mapa zasadnicza, ortofoto z geoportal.gov.pl) jako warstwy tła w mapach — bez pobierania danych.</t>
         </is>
       </c>
       <c r="H103" s="6" t="inlineStr">
@@ -11224,7 +11232,7 @@
       </c>
       <c r="G104" s="6" t="inlineStr">
         <is>
-          <t>Precyzyjna kontrola kto widzi co i co moze robic: administrator systemu -&gt; administrator bazy -&gt; edytor schematu -&gt; edytor tabeli -&gt; edytor pola. Bezpieczenstwo na kazdym poziomie.</t>
+          <t>Precyzyjna kontrola kto widzi co i co może robić: administrator systemu -&gt; administrator bazy -&gt; edytor schematu -&gt; edytor tabeli -&gt; edytor pola. Bezpieczeństwo na każdym poziomie.</t>
         </is>
       </c>
       <c r="H104" s="6" t="inlineStr">
@@ -11315,7 +11323,7 @@
       </c>
       <c r="G105" s="6" t="inlineStr">
         <is>
-          <t>Bezpieczne logowanie przez tokeny - sesja nie wygasa nieoczekiwanie, dane logowania nie sa przesylane przy kazdym zadaniu.</t>
+          <t>Bezpieczne logowanie przez tokeny — sesja nie wygasa nieoczekiwanie, dane logowania nie są przesyłane przy każdym zadaniu.</t>
         </is>
       </c>
       <c r="H105" s="6" t="inlineStr">
@@ -11406,7 +11414,7 @@
       </c>
       <c r="G106" s="6" t="inlineStr">
         <is>
-          <t>Dostep do systemu tylko z okreslonych adresow IP (np. siec wewnetrzna urzedu) - ochrona przed nieautoryzowanym dostepem z internetu.</t>
+          <t>Dostęp do systemu tylko z określonych adresów IP (np. siec wewnętrzna urzędu) — ochrona przed nieautoryzowanym dostępem z internetu.</t>
         </is>
       </c>
       <c r="H106" s="6" t="inlineStr">
@@ -11497,7 +11505,7 @@
       </c>
       <c r="G107" s="6" t="inlineStr">
         <is>
-          <t>Logowanie domenowe Active Directory - uzytkownicy uzywaja tych samych danych co do sieci firmowej, bez dodatkowych hasel GIS.</t>
+          <t>Logowanie domenowe Active Directory — użytkownicy używają tych samych danych co do sieci firmowej, bez dodatkowych haseł GIS.</t>
         </is>
       </c>
       <c r="H107" s="6" t="inlineStr">
@@ -11588,7 +11596,7 @@
       </c>
       <c r="G108" s="6" t="inlineStr">
         <is>
-          <t>Szyfrowanie komunikacji i tokenowe uwierzytelnianie - standard bezpieczenstwa dla aplikacji webowych. Spelnienie wymagan Krajowych Ram Interoperacyjnosci (KRI).</t>
+          <t>Szyfrowanie komunikacji i tokenowe uwierzytelnianie — standard bezpieczeństwa dla aplikacji webowych. Spełnienie wymagań Krajowych Ram Interoperacyjności (KRI).</t>
         </is>
       </c>
       <c r="H108" s="6" t="inlineStr">
@@ -11679,7 +11687,7 @@
       </c>
       <c r="G109" s="6" t="inlineStr">
         <is>
-          <t>Bezpieczenstwo danych realizowane na poziomie bazy Oracle - eliminuje ryzyko obejscia filtrow przez bezposredni dostep SQL.</t>
+          <t>Bezpieczeństwo danych realizowane na poziomie bazy Oracle — eliminuje ryzyko obejścia filtrów przez bezpośredni dostęp SQL.</t>
         </is>
       </c>
       <c r="H109" s="6" t="inlineStr">
@@ -11770,7 +11778,7 @@
       </c>
       <c r="G110" s="6" t="inlineStr">
         <is>
-          <t>Sledzenie kto, kiedy i co zmienil w danych. Raportowanie dostepu do danych osobowych - niezbedne dla compliance RODO.</t>
+          <t>Śledzenie kto, kiedy i co zmienił w danych. Raportowanie dostępu do danych osobowych — niezbedne dla compliance RODO.</t>
         </is>
       </c>
       <c r="H110" s="6" t="inlineStr">
@@ -11861,7 +11869,7 @@
       </c>
       <c r="G111" s="6" t="inlineStr">
         <is>
-          <t>Granularna kontrola dostepu do aplikacji webowych per uzytkownik lub rola - kazdy dzial/klient widzi tylko swoje aplikacje.</t>
+          <t>Granularna kontrola dostępu do aplikacji webowych per użytkownik lub rola — każdy dział/klient widzi tylko swoje aplikacje.</t>
         </is>
       </c>
       <c r="H111" s="6" t="inlineStr">
@@ -11952,7 +11960,7 @@
       </c>
       <c r="G112" s="6" t="inlineStr">
         <is>
-          <t>Mozliwosc ukrycia wrazliwych pol (np. PESEL, dane wlasciciela) dla okreslonych uzytkownikow - ochrona danych osobowych na poziomie API.</t>
+          <t>Możliwość ukrycia wrażliwych pol (np. PESEL, dane właściciela) dla określonych użytkowników — ochrona danych osobowych na poziomie API.</t>
         </is>
       </c>
       <c r="H112" s="6" t="inlineStr">
@@ -12043,7 +12051,7 @@
       </c>
       <c r="G113" s="6" t="inlineStr">
         <is>
-          <t>Graficzny panel do zarzadzania calym systemem - administratorzy nie musza edytowac plikow konfiguracyjnych ani pisac skryptow.</t>
+          <t>Graficzny panel do zarządzania całym systemem — administratorzy nie muszą edytować plików konfiguracyjnych ani pisać skryptów.</t>
         </is>
       </c>
       <c r="H113" s="6" t="inlineStr">
@@ -12134,7 +12142,7 @@
       </c>
       <c r="G114" s="6" t="inlineStr">
         <is>
-          <t>Uruchamianie, zatrzymywanie i konfigurowanie uslug mapowych przez prosty interfejs webowy - zarzadzanie bez dostepu SSH do serwera.</t>
+          <t>Uruchamianie, zatrzymywanie i konfigurowanie usług mapowych przez prosty interfejs webowy — zarządzanie bez dostępu SSH do serwera.</t>
         </is>
       </c>
       <c r="H114" s="6" t="inlineStr">
@@ -12225,7 +12233,7 @@
       </c>
       <c r="G115" s="6" t="inlineStr">
         <is>
-          <t>Dodawanie, testowanie i usuwanie polaczen z bazami danych - weryfikacja polaczenia w czasie rzeczywistym bez pisania kodu.</t>
+          <t>Dodawanie, testowanie i usuwanie połączeń z bazami danych — weryfikacja polaczenia w czasie rzeczywistym bez pisania kodu.</t>
         </is>
       </c>
       <c r="H115" s="6" t="inlineStr">
@@ -12316,7 +12324,7 @@
       </c>
       <c r="G116" s="6" t="inlineStr">
         <is>
-          <t>Tworzenie uzytkownikow, przypisywanie rol i uprawnien przez interfejs graficzny - bez SQL i skryptow.</t>
+          <t>Tworzenie użytkowników, przypisywanie rol i uprawnień przez interfejs graficzny — bez SQL i skryptów.</t>
         </is>
       </c>
       <c r="H116" s="6" t="inlineStr">
@@ -12407,7 +12415,7 @@
       </c>
       <c r="G117" s="6" t="inlineStr">
         <is>
-          <t>Podglad logow, statystyk uzycia i bledow w czasie rzeczywistym - szybka diagnostyka problemow bez analizowania plikow na serwerze.</t>
+          <t>Podgląd logów, statystyk użycia i błędów w czasie rzeczywistym — szybka diagnostyka problemów bez analizowania plików na serwerze.</t>
         </is>
       </c>
       <c r="H117" s="6" t="inlineStr">
@@ -12498,7 +12506,7 @@
       </c>
       <c r="G118" s="6" t="inlineStr">
         <is>
-          <t>Harmonogramowanie i zarzadzanie generowaniem kafelkow przez interfejs webowy - bez skryptow i linii polecen.</t>
+          <t>Harmonogramowanie i zarządzanie generowaniem kafli przez interfejs webowy — bez skryptów i linii poleceń.</t>
         </is>
       </c>
       <c r="H118" s="6" t="inlineStr">
@@ -12589,7 +12597,7 @@
       </c>
       <c r="G119" s="6" t="inlineStr">
         <is>
-          <t>Podglad warstwy lub uslugi bezposrednio w panelu admina - weryfikacja ze dane sa prawidlowe przed opublikowaniem dla uzytkownikow.</t>
+          <t>Podgląd warstwy lub usługi bezpośrednio w panelu admina — weryfikacja że dane są prawidłowe przed opublikowaniem dla użytkowników.</t>
         </is>
       </c>
       <c r="H119" s="6" t="inlineStr">
@@ -12680,7 +12688,7 @@
       </c>
       <c r="G120" s="6" t="inlineStr">
         <is>
-          <t>Uruchamianie, monitorowanie i zarzadzanie zadaniami geoprzetwarzania przez graficzny panel - bez CLI.</t>
+          <t>Uruchamianie, monitorowanie i zarządzanie zadaniami geoprzetwarzania przez graficzny panel — bez CLI.</t>
         </is>
       </c>
       <c r="H120" s="6" t="inlineStr">
@@ -12771,7 +12779,7 @@
       </c>
       <c r="G121" s="6" t="inlineStr">
         <is>
-          <t>Publikowanie i zarzadzanie aplikacjami webowymi przez panel admina - wdrazanie zmian bez dzialu IT.</t>
+          <t>Publikowanie i zarządzanie aplikacjami webowymi przez panel admina — wdrażanie zmian bez działu IT.</t>
         </is>
       </c>
       <c r="H121" s="6" t="inlineStr">
@@ -12862,7 +12870,7 @@
       </c>
       <c r="G122" s="6" t="inlineStr">
         <is>
-          <t>Topologiczna baza danych sieci (drogi, kanalizacja, sieci elektryczne) - podloze dla analiz sieciowych.</t>
+          <t>Topologiczna baza danych sieci (drogi, kanalizacja, sieci elektryczne) — podłoże dla analiz sieciowych.</t>
         </is>
       </c>
       <c r="H122" s="6" t="inlineStr">
@@ -12957,7 +12965,7 @@
       </c>
       <c r="G123" s="6" t="inlineStr">
         <is>
-          <t>Obliczanie obszarow dostepnych w X minut jazdy/marszu (izochory) - planowanie lokalizacji, analiza dostepnosci uslug, ewakuacja.</t>
+          <t>Obliczanie obszarów dostępnych w X minut jazdy/marszu (izochory) — planowanie lokalizacji, analiza dostępności usług, ewakuacja.</t>
         </is>
       </c>
       <c r="H123" s="6" t="inlineStr">
@@ -13052,7 +13060,7 @@
       </c>
       <c r="G124" s="6" t="inlineStr">
         <is>
-          <t>Wyznaczanie optymalnych tras (najkrotsza, najszybsza, z objazdem przeszkod) - logistyka, planowanie inspekcji terenowych, nawigacja.</t>
+          <t>Wyznaczanie optymalnych tras (najkrótsza, najszybsza, z objazdem przeszkód) — logistyka, planowanie inspekcji terenowych, nawigacja.</t>
         </is>
       </c>
       <c r="H124" s="6" t="inlineStr">
@@ -13147,7 +13155,7 @@
       </c>
       <c r="G125" s="6" t="inlineStr">
         <is>
-          <t>Automatyczna weryfikacja spojnosci sieci (wezly, polaczenia, kierunkowosc) - gwarancja poprawnosci analiz sieciowych.</t>
+          <t>Automatyczna weryfikacja spójności sieci (węzły, polaczenia, kierunkowość) — gwarancja poprawności analiz sieciowych.</t>
         </is>
       </c>
       <c r="H125" s="6" t="inlineStr">
@@ -13242,7 +13250,7 @@
       </c>
       <c r="G126" s="6" t="inlineStr">
         <is>
-          <t>Zaawansowane wizualizacje statystyczne: kartodiagramy (slupki per gmina na mapie) i kartogramy (mapa choropleth) - czytelna komunikacja danych dla decydentow.</t>
+          <t>Zaawansowane wizualizacje statystyczne: kartodiagramy (słupki per gmina na mapie) i kartogramy (mapa choropleth) — czytelna komunikacja danych dla decydentów.</t>
         </is>
       </c>
       <c r="H126" s="6" t="inlineStr">
@@ -13337,7 +13345,7 @@
       </c>
       <c r="G127" s="6" t="inlineStr">
         <is>
-          <t>Analiza skupisk i wzorow przestrzennych w danych (np. czy wypadki sa przypadkowe czy skupione w konkretnych miejscach) - wspomaganie decyzji opartych na danych.</t>
+          <t>Analiza skupisk i wzorów przestrzennych w danych (np. czy wypadki są przypadkowe czy skupione w konkretnych miejscach) — wspomaganie decyzji opartych na danych.</t>
         </is>
       </c>
       <c r="H127" s="6" t="inlineStr">
@@ -13432,7 +13440,7 @@
       </c>
       <c r="G128" s="6" t="inlineStr">
         <is>
-          <t>Dane dostepne przez API w standardowym formacie JSON/GeoJSON - integracja z dowolnym nowoczesnym systemem informatycznym i narzedzami open-source.</t>
+          <t>Dane dostępne przez API w standardowym formacie JSON/GeoJSON — integracja z dowolnym nowoczesnym systemem informatycznym i narzędziami open-source.</t>
         </is>
       </c>
       <c r="H128" s="6" t="inlineStr">
@@ -13523,7 +13531,7 @@
       </c>
       <c r="G129" s="6" t="inlineStr">
         <is>
-          <t>Mapy generowane jako obrazy PNG/JPG - gotowe do wklejenia w raporty, prezentacje PowerPoint, dokumenty Word.</t>
+          <t>Mapy generowane jako obrazy PNG/JPG — gotowe do wklejenia w raporty, prezentacje PowerPoint, dokumenty Word.</t>
         </is>
       </c>
       <c r="H129" s="6" t="inlineStr">
@@ -13614,7 +13622,7 @@
       </c>
       <c r="G130" s="6" t="inlineStr">
         <is>
-          <t>Eksport danych do KMZ/KML - otwieranie w Google Earth, Google My Maps, aplikacjach mobilnych.</t>
+          <t>Eksport danych do KMZ/KML — otwieranie w Google Earth, Google My Maps, aplikacjach mobilnych.</t>
         </is>
       </c>
       <c r="H130" s="6" t="inlineStr">
@@ -13705,7 +13713,7 @@
       </c>
       <c r="G131" s="6" t="inlineStr">
         <is>
-          <t>Eksport atrybutow do pliku CSV - analiza w Excelu, importowanie do systemow ERP/CRM, przetwarzanie w Pythonie/R.</t>
+          <t>Eksport atrybutów do pliku CSV — analiza w Excelu, importowanie do systemów ERP/CRM, przetwarzanie w Pythonie/R.</t>
         </is>
       </c>
       <c r="H131" s="6" t="inlineStr">
@@ -13796,7 +13804,7 @@
       </c>
       <c r="G132" s="6" t="inlineStr">
         <is>
-          <t>Format GeoPackage (jeden plik z wieloma warstwami) - standard do pracy offline w terenie i wymiany danych z QGIS.</t>
+          <t>Format GeoPackage (jeden plik z wieloma warstwami) — standard do pracy offline w terenie i wymiany danych z QGIS.</t>
         </is>
       </c>
       <c r="H132" s="6" t="inlineStr">
@@ -13887,7 +13895,7 @@
       </c>
       <c r="G133" s="6" t="inlineStr">
         <is>
-          <t>Kafelki wektorowe (PBF/MVT) - najszybszy format dla nowoczesnych aplikacji webowych renderujacych mapy po stronie klienta.</t>
+          <t>Kafle wektorowe (PBF/MVT) — najszybszy format dla nowoczesnych aplikacji webowych renderujacych mapy po stronie klienta.</t>
         </is>
       </c>
       <c r="H133" s="6" t="inlineStr">
@@ -13978,7 +13986,7 @@
       </c>
       <c r="G134" s="6" t="inlineStr">
         <is>
-          <t>Eksport do SQLite/SpatiaLite - lekka baza plikowa idealna dla aplikacji mobilnych i dystrybucji danych bez serwera.</t>
+          <t>Eksport do SQLite/SpatiaLite — lekka baza plikowa idealna dla aplikacji mobilnych i dystrybucji danych bez serwera.</t>
         </is>
       </c>
       <c r="H134" s="6" t="inlineStr">
@@ -14069,7 +14077,7 @@
       </c>
       <c r="G135" s="6" t="inlineStr">
         <is>
-          <t>Shapefile - klasyczny format wymiany z innymi systemami GIS, CAD i zewnetrznymi partnerami.</t>
+          <t>Shapefile — klasyczny format wymiany z innymi systemami GIS, CAD i zewnętrznymi partnerami.</t>
         </is>
       </c>
       <c r="H135" s="6" t="inlineStr">
@@ -14160,7 +14168,7 @@
       </c>
       <c r="G136" s="6" t="inlineStr">
         <is>
-          <t>Eksport modeli 3D (GLB/OBJ) - wizualizacja budynkow i infrastruktury w narzedzach 3D (Blender, Unity, przegladarka WebGL).</t>
+          <t>Eksport modeli 3D (GLB/OBJ) — wizualizacja budynków i infrastruktury w narzedzach 3D (Blender, Unity, przeglądarka WebGL).</t>
         </is>
       </c>
       <c r="H136" s="6" t="inlineStr">
@@ -14249,11 +14257,7 @@
           <t>Action Message Format – binarny format dla starszych klientów Flash/Flex.</t>
         </is>
       </c>
-      <c r="G137" s="6" t="inlineStr">
-        <is>
-          <t>Format AMF do specjalistycznych zastosowan 3D i druku przestrzennego.</t>
-        </is>
-      </c>
+      <c r="G137" s="6" t="n"/>
       <c r="H137" s="6" t="inlineStr">
         <is>
           <t>format</t>
@@ -14271,7 +14275,7 @@
       </c>
       <c r="O137" s="6" t="inlineStr">
         <is>
-          <t>potwierdzone</t>
+          <t>do weryfikacji</t>
         </is>
       </c>
       <c r="P137" s="6" t="inlineStr"/>
@@ -14307,7 +14311,11 @@
       <c r="AT137" s="6" t="inlineStr"/>
       <c r="AU137" s="6" t="inlineStr"/>
       <c r="AV137" s="6" t="inlineStr"/>
-      <c r="AW137" s="6" t="inlineStr"/>
+      <c r="AW137" s="6" t="inlineStr">
+        <is>
+          <t>Brak potwierdzenia w bazie wiedzy: zero wzmianek o AMF / Action Message Format w gp-knowledgebase (stan 2026-07-28). Udokumentowane wartości parametru f: html, json, pjson; dodatkowo PBF (pl.gispartner.imapserver.ags.pbf). Plik api/getstarted/output_formats.md jest pusty (0 B). Do potwierdzenia w kodzie: czy format jest nadal obsługiwany, czy wycofany.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
@@ -14342,7 +14350,7 @@
       </c>
       <c r="G138" s="6" t="inlineStr">
         <is>
-          <t>Podglad wynikow zapytan bezposrednio w przegladarce - szybkie testowanie i demonstracja danych bez instalowania klienta GIS.</t>
+          <t>Podgląd wyników zapytań bezpośrednio w przeglądarce — szybkie testowanie i demonstracja danych bez instalowania klienta GIS.</t>
         </is>
       </c>
       <c r="H138" s="6" t="inlineStr">
@@ -14431,7 +14439,11 @@
           <t>Bufory wokół obiektów.</t>
         </is>
       </c>
-      <c r="G139" s="6" t="inlineStr"/>
+      <c r="G139" s="6" t="inlineStr">
+        <is>
+          <t>Tworzenie stref ochronnych wokół obiektów (np. 100 m od drogi, 500 m od rzeki). Fundament analiz oddziaływania i planowania przestrzennego.</t>
+        </is>
+      </c>
       <c r="H139" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -14526,7 +14538,11 @@
           <t>Centroidy poligonów.</t>
         </is>
       </c>
-      <c r="G140" s="6" t="inlineStr"/>
+      <c r="G140" s="6" t="inlineStr">
+        <is>
+          <t>Wyznaczanie środków ciężkości poligonów — do etykiet na mapie, analiz położenia, markery zamiast pełnych poligonów.</t>
+        </is>
+      </c>
       <c r="H140" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -14621,7 +14637,11 @@
           <t>Długość, pole, wierzchołki, poprawność.</t>
         </is>
       </c>
-      <c r="G141" s="6" t="inlineStr"/>
+      <c r="G141" s="6" t="inlineStr">
+        <is>
+          <t>Automatyczne obliczanie długości, powierzchni, liczby wierzchołków i poprawności geometrii — podstawa kontroli jakości danych.</t>
+        </is>
+      </c>
       <c r="H141" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -14716,7 +14736,11 @@
           <t>Uproszczenie geometrii.</t>
         </is>
       </c>
-      <c r="G142" s="6" t="inlineStr"/>
+      <c r="G142" s="6" t="inlineStr">
+        <is>
+          <t>Upraszczanie skomplikowanych granic do prostszych kształtów — szybsze mapy przeglądowe, mniejsze pliki, lepsza czytelność.</t>
+        </is>
+      </c>
       <c r="H142" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -14811,7 +14835,11 @@
           <t>Podział linii wg max długości.</t>
         </is>
       </c>
-      <c r="G143" s="6" t="inlineStr"/>
+      <c r="G143" s="6" t="inlineStr">
+        <is>
+          <t>Podział długich linii na równe odcinki — przygotowanie sieci do analiz liniowych i interpolacji atrybutów.</t>
+        </is>
+      </c>
       <c r="H143" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -14906,7 +14934,11 @@
           <t>Podział poligonów wg liczby wierzchołków.</t>
         </is>
       </c>
-      <c r="G144" s="6" t="inlineStr"/>
+      <c r="G144" s="6" t="inlineStr">
+        <is>
+          <t>Dzielenie dużych poligonów na mniejsze części — optymalizacja zbiorów dla analiz przestrzennych i wydajności bazy.</t>
+        </is>
+      </c>
       <c r="H144" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15001,7 +15033,11 @@
           <t>Rozbicie multigeometrii na części.</t>
         </is>
       </c>
-      <c r="G145" s="6" t="inlineStr"/>
+      <c r="G145" s="6" t="inlineStr">
+        <is>
+          <t>Rozbijanie obiektów wieloczęściowych na pojedyncze — uporządkowanie danych przed analizą, eliminacja multigeometrii.</t>
+        </is>
+      </c>
       <c r="H145" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15096,7 +15132,11 @@
           <t>Punkt per wierzchołek geometrii.</t>
         </is>
       </c>
-      <c r="G146" s="6" t="inlineStr"/>
+      <c r="G146" s="6" t="inlineStr">
+        <is>
+          <t>Ekstrakcja wierzchołków geometrii jako osobnych punktów — analiza dokładności digitalizacji, generowanie siatek próbkowania.</t>
+        </is>
+      </c>
       <c r="H146" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15191,7 +15231,11 @@
           <t>Zaokrąglenie do siatki.</t>
         </is>
       </c>
-      <c r="G147" s="6" t="inlineStr"/>
+      <c r="G147" s="6" t="inlineStr">
+        <is>
+          <t>Wyrównywanie współrzędnych do siatki — normalizacja danych z różnych źródeł, eliminacja mikrobłędów topologicznych.</t>
+        </is>
+      </c>
       <c r="H147" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15286,7 +15330,11 @@
           <t>Przekształcenie przez macierz afiniczną.</t>
         </is>
       </c>
-      <c r="G148" s="6" t="inlineStr"/>
+      <c r="G148" s="6" t="inlineStr">
+        <is>
+          <t>Geometryczne przekształcenia obiektów (rotacja, skalowanie, przesunięcie) — dostosowanie danych do docelowego układu przestrzennego.</t>
+        </is>
+      </c>
       <c r="H148" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15381,7 +15429,11 @@
           <t>Przeliczenie do nowego CRS.</t>
         </is>
       </c>
-      <c r="G149" s="6" t="inlineStr"/>
+      <c r="G149" s="6" t="inlineStr">
+        <is>
+          <t>Zmiana układu współrzędnych całych zbiorów danych — migracja między PUWG 92, 2000, WGS84, web Mercator.</t>
+        </is>
+      </c>
       <c r="H149" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15476,7 +15528,11 @@
           <t>X↔Y w geometrii.</t>
         </is>
       </c>
-      <c r="G150" s="6" t="inlineStr"/>
+      <c r="G150" s="6" t="inlineStr">
+        <is>
+          <t>Zamiana kolejności X/Y — naprawa danych z błędną kolejnością współrzędnych bez ręcznej edycji.</t>
+        </is>
+      </c>
       <c r="H150" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15571,7 +15627,11 @@
           <t>Najmniejsze koło otaczające zbiór.</t>
         </is>
       </c>
-      <c r="G151" s="6" t="inlineStr"/>
+      <c r="G151" s="6" t="inlineStr">
+        <is>
+          <t>Generowanie najmniejszego okręgu otaczającego obiekt — analiza zasięgu, kompaktowości kształtów.</t>
+        </is>
+      </c>
       <c r="H151" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15666,7 +15726,11 @@
           <t>Generowanie punktów wewnątrz geometrii.</t>
         </is>
       </c>
-      <c r="G152" s="6" t="inlineStr"/>
+      <c r="G152" s="6" t="inlineStr">
+        <is>
+          <t>Tworzenie siatki punktów próbkowania wewnątrz poligonów — planowanie inwentaryzacji terenowej, rozmieszczenie pomiarów.</t>
+        </is>
+      </c>
       <c r="H152" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15761,7 +15825,11 @@
           <t>Punkty z listy współrzędnych (x,y,CRS).</t>
         </is>
       </c>
-      <c r="G153" s="6" t="inlineStr"/>
+      <c r="G153" s="6" t="inlineStr">
+        <is>
+          <t>Import lokalizacji z tabeli (x, y, CRS) jako warstwa punktowa — geokodowanie współrzędnymi zamiast adresami.</t>
+        </is>
+      </c>
       <c r="H153" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15856,7 +15924,11 @@
           <t>Iloczyn przestrzenny zbiorów.</t>
         </is>
       </c>
-      <c r="G154" s="6" t="inlineStr"/>
+      <c r="G154" s="6" t="inlineStr">
+        <is>
+          <t>Obliczanie części wspólnej dwóch warstw — np. działki w strefie zalewowej, tereny w zasięgu planowanej inwestycji.</t>
+        </is>
+      </c>
       <c r="H154" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -15951,7 +16023,11 @@
           <t>Zbiór 1 minus część wspólna z 2.</t>
         </is>
       </c>
-      <c r="G155" s="6" t="inlineStr"/>
+      <c r="G155" s="6" t="inlineStr">
+        <is>
+          <t>Odejmowanie geometrii — co pozostaje po wyjęciu jednego zbioru (np. tereny niezabudowane = gmina minus zabudowa).</t>
+        </is>
+      </c>
       <c r="H155" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16046,7 +16122,11 @@
           <t>Obiekty wyłącznie z jednego ze zbiorów.</t>
         </is>
       </c>
-      <c r="G156" s="6" t="inlineStr"/>
+      <c r="G156" s="6" t="inlineStr">
+        <is>
+          <t>Obiekty które są tylko w jednym ze zbiorów — wykrywanie zmian między dwoma wersjami danych ewidencyjnych.</t>
+        </is>
+      </c>
       <c r="H156" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16141,7 +16221,11 @@
           <t>Pocięcie zbioru 1 geometrią zbioru 2.</t>
         </is>
       </c>
-      <c r="G157" s="6" t="inlineStr"/>
+      <c r="G157" s="6" t="inlineStr">
+        <is>
+          <t>Przecinanie obiektów przez inną linię lub granice — podział działek przez planowaną drogę lub granicę administracyjną.</t>
+        </is>
+      </c>
       <c r="H157" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16236,7 +16320,11 @@
           <t>Clip do zasięgu zbioru 2.</t>
         </is>
       </c>
-      <c r="G158" s="6" t="inlineStr"/>
+      <c r="G158" s="6" t="inlineStr">
+        <is>
+          <t>Przycinanie warstwy do obszaru zainteresowania — ograniczenie danych do granic gminy, powiatu lub projektu.</t>
+        </is>
+      </c>
       <c r="H158" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16331,7 +16419,11 @@
           <t>Połączenie wielu zbiorów w jeden.</t>
         </is>
       </c>
-      <c r="G159" s="6" t="inlineStr"/>
+      <c r="G159" s="6" t="inlineStr">
+        <is>
+          <t>Łączenie wielu zbiorów danych w jeden — integracja danych z różnych gmin lub źródeł w jeden zbiór roboczy.</t>
+        </is>
+      </c>
       <c r="H159" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16426,7 +16518,11 @@
           <t>Dissolve z opcjonalnymi statystykami.</t>
         </is>
       </c>
-      <c r="G160" s="6" t="inlineStr"/>
+      <c r="G160" s="6" t="inlineStr">
+        <is>
+          <t>Scalanie obiektów o tych samych atrybutach w jeden — np. granice gmin scalane do powiatów, odcinki drogi w jeden przebieg.</t>
+        </is>
+      </c>
       <c r="H160" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16521,7 +16617,11 @@
           <t>Kopia zbioru (z filtracją).</t>
         </is>
       </c>
-      <c r="G161" s="6" t="inlineStr"/>
+      <c r="G161" s="6" t="inlineStr">
+        <is>
+          <t>Tworzenie kopii warstwy lub wybranego podzbioru — archiwizacja stanu danych przed edycją lub eksportem.</t>
+        </is>
+      </c>
       <c r="H161" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16616,7 +16716,11 @@
           <t>Filtr wg warunków atrybutowych.</t>
         </is>
       </c>
-      <c r="G162" s="6" t="inlineStr"/>
+      <c r="G162" s="6" t="inlineStr">
+        <is>
+          <t>Wybór obiektów spełniających warunek atrybutowy — filtrowanie zbioru do analizy bez usuwania pozostałych danych.</t>
+        </is>
+      </c>
       <c r="H162" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16711,7 +16815,11 @@
           <t>Obiekty bez części wspólnej z zbiorem 2.</t>
         </is>
       </c>
-      <c r="G163" s="6" t="inlineStr"/>
+      <c r="G163" s="6" t="inlineStr">
+        <is>
+          <t>Obiekty które NIE mają części wspólnej z innym zbiorem — np. budynki poza strefami ochronnymi.</t>
+        </is>
+      </c>
       <c r="H163" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16806,7 +16914,11 @@
           <t>Obiekty z częścią wspólną z zbiorem 2.</t>
         </is>
       </c>
-      <c r="G164" s="6" t="inlineStr"/>
+      <c r="G164" s="6" t="inlineStr">
+        <is>
+          <t>Obiekty mające część wspólną z innym zbiorem — np. budynki na terenach zagrożeń powodziowych.</t>
+        </is>
+      </c>
       <c r="H164" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16901,7 +17013,11 @@
           <t>Usunięcie zduplikowanych punktów.</t>
         </is>
       </c>
-      <c r="G165" s="6" t="inlineStr"/>
+      <c r="G165" s="6" t="inlineStr">
+        <is>
+          <t>Eliminacja zduplikowanych wierzchołków geometrii — czyszczenie danych z powtarzającymi się punktami.</t>
+        </is>
+      </c>
       <c r="H165" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -16996,7 +17112,11 @@
           <t>Usunięcie wg kryterium atrybutowego.</t>
         </is>
       </c>
-      <c r="G166" s="6" t="inlineStr"/>
+      <c r="G166" s="6" t="inlineStr">
+        <is>
+          <t>Usuwanie wybranych obiektów z warstwy na podstawie warunku atrybutowego — czyszczenie danych niespełniających kryterium jakości.</t>
+        </is>
+      </c>
       <c r="H166" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17091,7 +17211,11 @@
           <t>Usunięcie obiektów z częścią wspólną z 2.</t>
         </is>
       </c>
-      <c r="G167" s="6" t="inlineStr"/>
+      <c r="G167" s="6" t="inlineStr">
+        <is>
+          <t>Usuwanie obiektów nakładających się z inną warstwą — eliminacja obiektów w strefach wykluczenia.</t>
+        </is>
+      </c>
       <c r="H167" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17186,7 +17310,11 @@
           <t>Join przez relację przestrzenną.</t>
         </is>
       </c>
-      <c r="G168" s="6" t="inlineStr"/>
+      <c r="G168" s="6" t="inlineStr">
+        <is>
+          <t>Automatyczne przypisanie atrybutów z jednej warstwy do drugiej na podstawie położenia — np. nazwa gminy do każdego budynku, numer działki do adresu.</t>
+        </is>
+      </c>
       <c r="H168" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17281,7 +17409,11 @@
           <t>Join przez wspólny klucz.</t>
         </is>
       </c>
-      <c r="G169" s="6" t="inlineStr"/>
+      <c r="G169" s="6" t="inlineStr">
+        <is>
+          <t>Łączenie danych tabelarycznych (CSV, XLS) z warstwa przestrzenna przez wspólny klucz — wzbogacenie geometrii o dane statystyczne.</t>
+        </is>
+      </c>
       <c r="H169" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17376,7 +17508,11 @@
           <t>Sum/avg/min/max pkt/lin w poligonach.</t>
         </is>
       </c>
-      <c r="G170" s="6" t="inlineStr"/>
+      <c r="G170" s="6" t="inlineStr">
+        <is>
+          <t>Obliczanie statystyk (suma, średnia, min, max) dla obiektów wewnątrz poligonów — np. średnia wysokość budynków per działka.</t>
+        </is>
+      </c>
       <c r="H170" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17471,7 +17607,11 @@
           <t>Wyrażenia matematyczne na atrybutach.</t>
         </is>
       </c>
-      <c r="G171" s="6" t="inlineStr"/>
+      <c r="G171" s="6" t="inlineStr">
+        <is>
+          <t>Masowe wyliczanie i aktualizacja wartości pól na podstawie wyrażeń matematycznych — przeliczenia, kategorie, wskaźniki dla całego zbioru naraz.</t>
+        </is>
+      </c>
       <c r="H171" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17566,7 +17706,11 @@
           <t>Gęstość pkt w poligonach referencyjnych.</t>
         </is>
       </c>
-      <c r="G172" s="6" t="inlineStr"/>
+      <c r="G172" s="6" t="inlineStr">
+        <is>
+          <t>Wizualizacja gęstości zjawisk punktowych w poligonach referencyjnych — identyfikacja hot spotów incydentów, zgłoszeń, inwestycji.</t>
+        </is>
+      </c>
       <c r="H172" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17661,7 +17805,11 @@
           <t>Najbliższy obiekt z odległością.</t>
         </is>
       </c>
-      <c r="G173" s="6" t="inlineStr"/>
+      <c r="G173" s="6" t="inlineStr">
+        <is>
+          <t>Wyznaczanie najbliższego obiektu i odległości do niego dla każdego elementu — analiza sąsiedztwa, dostępność usług.</t>
+        </is>
+      </c>
       <c r="H173" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17756,7 +17904,11 @@
           <t>Tesselacja Woronoja z wierzchołków.</t>
         </is>
       </c>
-      <c r="G174" s="6" t="inlineStr"/>
+      <c r="G174" s="6" t="inlineStr">
+        <is>
+          <t>Generowanie obszarów wpływu wokół punktów — strefy obsługi placówek, zasięg stacji, obszary Thiessena.</t>
+        </is>
+      </c>
       <c r="H174" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17851,7 +18003,11 @@
           <t>Punkt = mediana współrzędnych.</t>
         </is>
       </c>
-      <c r="G175" s="6" t="inlineStr"/>
+      <c r="G175" s="6" t="inlineStr">
+        <is>
+          <t>Wyznaczanie optymalnego punktu centralnego minimalizującego odległości — optymalna lokalizacja magazynu, centrum zdarzeń.</t>
+        </is>
+      </c>
       <c r="H175" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -17946,7 +18102,11 @@
           <t>Identyfikacja skupisk przestrzennych.</t>
         </is>
       </c>
-      <c r="G176" s="6" t="inlineStr"/>
+      <c r="G176" s="6" t="inlineStr">
+        <is>
+          <t>Automatyczne wykrywanie skupisk przestrzennych w danych punktowych — identyfikacja hot spotów wypadków, ognisk chorob, koncentracji inwestycji.</t>
+        </is>
+      </c>
       <c r="H176" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18041,7 +18201,11 @@
           <t>Liczba obiektów pkt/lin wewnątrz poligonów.</t>
         </is>
       </c>
-      <c r="G177" s="6" t="inlineStr"/>
+      <c r="G177" s="6" t="inlineStr">
+        <is>
+          <t>Zliczanie punktów i linii wewnątrz poligonów — liczba budynków per działka, incydenty per rejon, klienci per obszar sprzedaży.</t>
+        </is>
+      </c>
       <c r="H177" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18136,7 +18300,11 @@
           <t>Cieniowanie reliefu z DEM.</t>
         </is>
       </c>
-      <c r="G178" s="6" t="inlineStr"/>
+      <c r="G178" s="6" t="inlineStr">
+        <is>
+          <t>Cieniowanie rzeźby terenu z modelu wysokościowego (DEM) — czytelna wizualizacja ukształtowania terenu na mapie.</t>
+        </is>
+      </c>
       <c r="H178" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18231,7 +18399,11 @@
           <t>Mapa spadków z DEM.</t>
         </is>
       </c>
-      <c r="G179" s="6" t="inlineStr"/>
+      <c r="G179" s="6" t="inlineStr">
+        <is>
+          <t>Mapa nachyleń stoku z DEM — analiza zagrożenia osuwiskowego, dobór użytków rolnych, planowanie infrastruktury.</t>
+        </is>
+      </c>
       <c r="H179" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18326,7 +18498,11 @@
           <t>Przeliczenie CRS rastra.</t>
         </is>
       </c>
-      <c r="G180" s="6" t="inlineStr"/>
+      <c r="G180" s="6" t="inlineStr">
+        <is>
+          <t>Zmiana układu współrzędnych rastra — dostosowanie zdjęć lotniczych lub NMT do układu mapy projektowej.</t>
+        </is>
+      </c>
       <c r="H180" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18421,7 +18597,11 @@
           <t>Zmiana rozdzielczości przestrzennej.</t>
         </is>
       </c>
-      <c r="G181" s="6" t="inlineStr"/>
+      <c r="G181" s="6" t="inlineStr">
+        <is>
+          <t>Zmiana rozdzielczości piksela rastra — optymalizacja dla wydajności przy dużych zbiorach lub dokładności przy analizach precyzyjnych.</t>
+        </is>
+      </c>
       <c r="H181" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18516,7 +18696,11 @@
           <t>Przycięcie do poligonu/bbox.</t>
         </is>
       </c>
-      <c r="G182" s="6" t="inlineStr"/>
+      <c r="G182" s="6" t="inlineStr">
+        <is>
+          <t>Wycinanie fragmentu rastra do obszaru zainteresowania — ograniczenie dużego NMT lub ortofoto do obszaru projektu.</t>
+        </is>
+      </c>
       <c r="H182" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18611,7 +18795,11 @@
           <t>Mozaikowanie wielu rastrów.</t>
         </is>
       </c>
-      <c r="G183" s="6" t="inlineStr"/>
+      <c r="G183" s="6" t="inlineStr">
+        <is>
+          <t>Łączenie wielu rastrów w mozaikę — jednolity NMT lub ortofoto z kilku arkuszy lub lotów.</t>
+        </is>
+      </c>
       <c r="H183" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18706,7 +18894,11 @@
           <t>Poligon/linia → raster.</t>
         </is>
       </c>
-      <c r="G184" s="6" t="inlineStr"/>
+      <c r="G184" s="6" t="inlineStr">
+        <is>
+          <t>Konwersja poligonów i linii na raster — przygotowanie danych wektorowych do analiz rastrowych.</t>
+        </is>
+      </c>
       <c r="H184" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18801,7 +18993,11 @@
           <t>Warstwa wektorowa → raster.</t>
         </is>
       </c>
-      <c r="G185" s="6" t="inlineStr"/>
+      <c r="G185" s="6" t="inlineStr">
+        <is>
+          <t>Tworzenie rastra na podstawie wartości atrybutów warstwy wektorowej — np. mapa bonitacji gleb jako raster z wartości atrybutu.</t>
+        </is>
+      </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18896,7 +19092,11 @@
           <t>Raster → poligony.</t>
         </is>
       </c>
-      <c r="G186" s="6" t="inlineStr"/>
+      <c r="G186" s="6" t="inlineStr">
+        <is>
+          <t>Konwersja rastra klasyfikowanego na warstwę wektorową — ekstrakcja obszarów z satelitarnej klasyfikacji pokrycia terenu.</t>
+        </is>
+      </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -18991,7 +19191,11 @@
           <t>Punkt per piksel z wartością.</t>
         </is>
       </c>
-      <c r="G187" s="6" t="inlineStr"/>
+      <c r="G187" s="6" t="inlineStr">
+        <is>
+          <t>Konwersja każdego piksela rastra na punkt z wartością — próbkowanie wartości wysokościowych lub spektralnych.</t>
+        </is>
+      </c>
       <c r="H187" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19086,7 +19290,11 @@
           <t>Kontury/izolinie z rastra.</t>
         </is>
       </c>
-      <c r="G188" s="6" t="inlineStr"/>
+      <c r="G188" s="6" t="inlineStr">
+        <is>
+          <t>Generowanie poziomic i izolinii z rastra — poziomice z NMT, izobary z modelu meteorologicznego, izolinie hałasu.</t>
+        </is>
+      </c>
       <c r="H188" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19181,7 +19389,11 @@
           <t>Min, max, mean, std, histogram.</t>
         </is>
       </c>
-      <c r="G189" s="6" t="inlineStr"/>
+      <c r="G189" s="6" t="inlineStr">
+        <is>
+          <t>Obliczanie statystyk pikselowych (min, max, średnia, odch. std.) — analiza zakresu wartości NMT lub danych pomiarowych.</t>
+        </is>
+      </c>
       <c r="H189" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19276,7 +19488,11 @@
           <t>Zasięg danych i obszary NoData.</t>
         </is>
       </c>
-      <c r="G190" s="6" t="inlineStr"/>
+      <c r="G190" s="6" t="inlineStr">
+        <is>
+          <t>Analiza zasięgu danych rastrowych i obszarów bez danych — kontrola kompletności pokrycia przed analizą.</t>
+        </is>
+      </c>
       <c r="H190" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19371,7 +19587,11 @@
           <t>SHP/GeoJSON/GPKG/CSV/GDB → baza.</t>
         </is>
       </c>
-      <c r="G191" s="6" t="inlineStr"/>
+      <c r="G191" s="6" t="inlineStr">
+        <is>
+          <t>Automatyczny import danych z plików (SHP, GeoJSON, GPKG, CSV, GDB) do bazy — bez ręcznego ładowania przez narzędzia bazodanowe.</t>
+        </is>
+      </c>
       <c r="H191" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19466,7 +19686,11 @@
           <t>Inspekcja struktury przed importem.</t>
         </is>
       </c>
-      <c r="G192" s="6" t="inlineStr"/>
+      <c r="G192" s="6" t="inlineStr">
+        <is>
+          <t>Inspekcja struktury i zawartość pliku przed importem — weryfikacja pol, typów i układu bez otwierania pliku w GIS.</t>
+        </is>
+      </c>
       <c r="H192" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19561,7 +19785,11 @@
           <t>Nowa tabela w bazie danych.</t>
         </is>
       </c>
-      <c r="G193" s="6" t="inlineStr"/>
+      <c r="G193" s="6" t="inlineStr">
+        <is>
+          <t>Programowe tworzenie nowej tabeli w bazie danych — automatyzacja tworzenia struktur w procesach ETL.</t>
+        </is>
+      </c>
       <c r="H193" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19656,7 +19884,11 @@
           <t>Usunięcie schematu z tabelami.</t>
         </is>
       </c>
-      <c r="G194" s="6" t="inlineStr"/>
+      <c r="G194" s="6" t="inlineStr">
+        <is>
+          <t>Usuniecie schematu z wszystkimi tabelami — czyszczenie środowisk testowych i tymczasowych zbiorów roboczych.</t>
+        </is>
+      </c>
       <c r="H194" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19751,7 +19983,11 @@
           <t>Usunięcie wybranej tabeli.</t>
         </is>
       </c>
-      <c r="G195" s="6" t="inlineStr"/>
+      <c r="G195" s="6" t="inlineStr">
+        <is>
+          <t>Usuniecie wybranej tabeli z bazy — porządkowanie po zakończeniu projektu lub po zastąpieniu nowszymi danymi.</t>
+        </is>
+      </c>
       <c r="H195" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19846,7 +20082,11 @@
           <t>Zapytanie jako zadanie GP.</t>
         </is>
       </c>
-      <c r="G196" s="6" t="inlineStr"/>
+      <c r="G196" s="6" t="inlineStr">
+        <is>
+          <t>Wykonanie zapytania do danych jako zadanie GP — użycie pełnej logiki query (WHERE, statystyki, joins) w kontekście geoprzetwarzania.</t>
+        </is>
+      </c>
       <c r="H196" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -19941,7 +20181,11 @@
           <t>Mozaika z zestawu rastrów.</t>
         </is>
       </c>
-      <c r="G197" s="6" t="inlineStr"/>
+      <c r="G197" s="6" t="inlineStr">
+        <is>
+          <t>Tworzenie katalogu mozaiki rastrowej z zestawu plików — organizacja dużych kolekcji zdjęć do efektywnego serwowania.</t>
+        </is>
+      </c>
       <c r="H197" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -20036,7 +20280,11 @@
           <t>Import gotowej mozaiki.</t>
         </is>
       </c>
-      <c r="G198" s="6" t="inlineStr"/>
+      <c r="G198" s="6" t="inlineStr">
+        <is>
+          <t>Import gotowej mozaiki rastrowej do systemu iMapServer — szybkie udostępnianie dużych zbiorów zdjęć bez ponownego przetwarzania.</t>
+        </is>
+      </c>
       <c r="H198" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -20131,7 +20379,11 @@
           <t>Wsadowe ładowanie przez kursory DB.</t>
         </is>
       </c>
-      <c r="G199" s="6" t="inlineStr"/>
+      <c r="G199" s="6" t="inlineStr">
+        <is>
+          <t>Wsadowe ładowanie danych przez kursory bazodanowe — wysokowydajny import dużych zbiorów bez overhead'u REST API.</t>
+        </is>
+      </c>
       <c r="H199" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -20226,7 +20478,11 @@
           <t>Konwersja przez kursory DB.</t>
         </is>
       </c>
-      <c r="G200" s="6" t="inlineStr"/>
+      <c r="G200" s="6" t="inlineStr">
+        <is>
+          <t>Konwersja danych przez kursory bazodanowe — transformacja i przepisywanie dużych zbiorów między strukturami.</t>
+        </is>
+      </c>
       <c r="H200" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -20321,7 +20577,11 @@
           <t>Pakiet kafli wektorowych (.vtpk).</t>
         </is>
       </c>
-      <c r="G201" s="6" t="inlineStr"/>
+      <c r="G201" s="6" t="inlineStr">
+        <is>
+          <t>Tworzenie pakietu kafli wektorowych (.vtpk) — offline lub CDN-ready kafle dla aplikacji mobilnych i portal'i bez serwera.</t>
+        </is>
+      </c>
       <c r="H201" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -20416,7 +20676,11 @@
           <t>Pakiet scen 3D (.slpk).</t>
         </is>
       </c>
-      <c r="G202" s="6" t="inlineStr"/>
+      <c r="G202" s="6" t="inlineStr">
+        <is>
+          <t>Tworzenie pakietu scen 3D (.slpk) — offline-capable modele 3D miast i terenu dla SceneViewer.</t>
+        </is>
+      </c>
       <c r="H202" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>
@@ -20511,7 +20775,11 @@
           <t>Linear Referencing System: kalibracja, pomiar, zdarzenia na sieci.</t>
         </is>
       </c>
-      <c r="G203" s="6" t="inlineStr"/>
+      <c r="G203" s="6" t="inlineStr">
+        <is>
+          <t>Kalibracja tras, pomiar odległości na sieci, lokalizacja zdarzeń po kilometrażu (Linear Referencing) — obowiązek w systemach zarządzania drogami i sieciami.</t>
+        </is>
+      </c>
       <c r="H203" s="6" t="inlineStr">
         <is>
           <t>zadanie GP</t>

</xml_diff>